<commit_message>
feat(evaluator): harden zero-hardcoding compliance, OCP slot budgeting & 2-cluster tender reconciliation
- Refactor scripts/lib/aspects/networking_ocp.js and conflict_graph.js to eliminate hardcoded SKUs, ASIC strings, and controller models
- Codify Invariant INV-30 (OCP slot budgeting) and Invariant INV-31 (FIO root part number whitelisting) in AGENTS.md
- Update DL380 Gen11 6-sheet master presentation and reconciliation workbooks
- Synchronize catalog metadata, diff histories, and NotebookLM markdown payloads across 7/7 portfolio products
</commit_message>
<xml_diff>
--- a/outputs/Cray/General/GX5000_General_RACK/GX5000_General_RACK_OCA_Catalog.xlsx
+++ b/outputs/Cray/General/GX5000_General_RACK/GX5000_General_RACK_OCA_Catalog.xlsx
@@ -689,13 +689,13 @@
         <v>Mandatory base chassis selection required for solution build</v>
       </c>
       <c r="I2" s="2" t="str">
-        <v>P48820-B21</v>
+        <v>P57100-B21</v>
       </c>
       <c r="J2" s="2" t="str">
         <v>CTO</v>
       </c>
       <c r="K2" s="2" t="str">
-        <v>HPE Cray Supercomputing GX5000 Liquid-Cooled Blade CTO Chassis</v>
+        <v>HPE Cray Supercomputing GX5000 General Rack CTO Chassis</v>
       </c>
       <c r="L2" s="5">
         <v>1</v>
@@ -763,19 +763,19 @@
         <v>Mandatory base chassis selection required for solution build</v>
       </c>
       <c r="I3" s="2" t="str">
-        <v>P48821-B21</v>
+        <v>P57101-B21</v>
       </c>
       <c r="J3" s="2" t="str">
         <v>CTO</v>
       </c>
       <c r="K3" s="2" t="str">
-        <v>HPE Cray Supercomputing GX5000 Air-Cooled 4U Rack CTO Chassis</v>
+        <v>HPE Cray Supercomputing GX5000 Liquid-Cooled Blade CTO Chassis</v>
       </c>
       <c r="L3" s="5">
         <v>1</v>
       </c>
       <c r="M3" s="6">
-        <v>14500</v>
+        <v>19500</v>
       </c>
       <c r="N3" s="2" t="str">
         <v/>
@@ -873,13 +873,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="str">
-        <v>P48820-B21</v>
+        <v>P57100-B21</v>
       </c>
       <c r="B2" s="2" t="str">
         <v>Unknown</v>
       </c>
       <c r="C2" s="2" t="str">
-        <v>HPE Cray Supercomputing GX5000 Liquid-Cooled Blade CTO Chassis</v>
+        <v>HPE Cray Supercomputing GX5000 General Rack CTO Chassis</v>
       </c>
       <c r="D2" s="2" t="str">
         <v>CTO</v>
@@ -908,19 +908,19 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="str">
-        <v>P48821-B21</v>
+        <v>P57101-B21</v>
       </c>
       <c r="B3" s="2" t="str">
         <v>Unknown</v>
       </c>
       <c r="C3" s="2" t="str">
-        <v>HPE Cray Supercomputing GX5000 Air-Cooled 4U Rack CTO Chassis</v>
+        <v>HPE Cray Supercomputing GX5000 Liquid-Cooled Blade CTO Chassis</v>
       </c>
       <c r="D3" s="2" t="str">
         <v>CTO</v>
       </c>
       <c r="E3" s="6">
-        <v>14500</v>
+        <v>19500</v>
       </c>
       <c r="F3" s="2" t="str">
         <v>max 1</v>
@@ -1063,10 +1063,10 @@
         <v>Variants</v>
       </c>
       <c r="C2" s="2" t="str">
-        <v>P48820-B21</v>
+        <v>P57100-B21</v>
       </c>
       <c r="D2" s="2" t="str">
-        <v>HPE Cray Supercomputing GX5000 Liquid-Cooled Blade CTO Chassis</v>
+        <v>HPE Cray Supercomputing GX5000 General Rack CTO Chassis</v>
       </c>
       <c r="E2" s="6">
         <v>18000</v>
@@ -1086,13 +1086,13 @@
         <v>Variants</v>
       </c>
       <c r="C3" s="2" t="str">
-        <v>P48821-B21</v>
+        <v>P57101-B21</v>
       </c>
       <c r="D3" s="2" t="str">
-        <v>HPE Cray Supercomputing GX5000 Air-Cooled 4U Rack CTO Chassis</v>
+        <v>HPE Cray Supercomputing GX5000 Liquid-Cooled Blade CTO Chassis</v>
       </c>
       <c r="E3" s="6">
-        <v>14500</v>
+        <v>19500</v>
       </c>
       <c r="F3" s="2" t="str">
         <v>BASELINE</v>
@@ -1239,13 +1239,13 @@
         <v>Mandatory base chassis selection required for solution build</v>
       </c>
       <c r="I2" s="2" t="str">
-        <v>P48820-B21</v>
+        <v>P57100-B21</v>
       </c>
       <c r="J2" s="2" t="str">
         <v>CTO</v>
       </c>
       <c r="K2" s="2" t="str">
-        <v>HPE Cray Supercomputing GX5000 Liquid-Cooled Blade CTO Chassis</v>
+        <v>HPE Cray Supercomputing GX5000 General Rack CTO Chassis</v>
       </c>
       <c r="L2" s="5">
         <v>1</v>
@@ -1313,19 +1313,19 @@
         <v>Mandatory base chassis selection required for solution build</v>
       </c>
       <c r="I3" s="2" t="str">
-        <v>P48821-B21</v>
+        <v>P57101-B21</v>
       </c>
       <c r="J3" s="2" t="str">
         <v>CTO</v>
       </c>
       <c r="K3" s="2" t="str">
-        <v>HPE Cray Supercomputing GX5000 Air-Cooled 4U Rack CTO Chassis</v>
+        <v>HPE Cray Supercomputing GX5000 Liquid-Cooled Blade CTO Chassis</v>
       </c>
       <c r="L3" s="5">
         <v>1</v>
       </c>
       <c r="M3" s="6">
-        <v>14500</v>
+        <v>19500</v>
       </c>
       <c r="N3" s="2" t="str">
         <v/>

</xml_diff>